<commit_message>
Changed data for registration
</commit_message>
<xml_diff>
--- a/DEMOWEBSHOP/TestData/TestData.xlsx
+++ b/DEMOWEBSHOP/TestData/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vithy\Desktop\Expleo\AUTOMATIONPROJECT\DEMOWEBSHOP\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96FD8955-64BA-41C7-B6D0-EFC5040027D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6010BF32-394C-4CAA-AAB1-13A8A029CCE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="732" yWindow="732" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -70,10 +70,10 @@
     <t>john123</t>
   </si>
   <si>
-    <t>vithyakm12345@gmail.com</t>
-  </si>
-  <si>
-    <t>johnkm12345@gmail.com</t>
+    <t>vithyakm123456@gmail.com</t>
+  </si>
+  <si>
+    <t>johnkm123456@gmail.com</t>
   </si>
 </sst>
 </file>

</xml_diff>